<commit_message>
fix: exclude global SUPER_ADMIN platform accounts from school staff registry
</commit_message>
<xml_diff>
--- a/new_passwords.xlsx
+++ b/new_passwords.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/Documents/Tech_projects/report_automation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03E43B53-A2C1-2F46-9574-6798C828E773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC64B575-D3ED-E34F-8068-ACA1029CCB90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="33600" windowHeight="20380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3600,14 +3600,14 @@
     <t>admin</t>
   </si>
   <si>
-    <t>Nacho-RM9P6VWE</t>
+    <t>Admin123456!</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -3624,10 +3624,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Geist Mono"/>
+      <sz val="13"/>
+      <color rgb="FFD7BA7D"/>
+      <name val="Menlo"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -4011,13 +4011,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="4" width="35.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4037,7 +4037,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>7</v>
       </c>
@@ -4065,12 +4065,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G109"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="43.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4093,7 +4093,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -4116,7 +4116,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -4139,7 +4139,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -4162,7 +4162,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -4185,7 +4185,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -4208,7 +4208,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -4231,7 +4231,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -4254,7 +4254,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -4277,7 +4277,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -4300,7 +4300,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -4323,7 +4323,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -4346,7 +4346,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -4369,7 +4369,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -4392,7 +4392,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -4415,7 +4415,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -4438,7 +4438,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -4461,7 +4461,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -4484,7 +4484,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>8</v>
       </c>
@@ -4507,7 +4507,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>8</v>
       </c>
@@ -4530,7 +4530,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -4553,7 +4553,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>8</v>
       </c>
@@ -4576,7 +4576,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -4599,7 +4599,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>8</v>
       </c>
@@ -4622,7 +4622,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>8</v>
       </c>
@@ -4645,7 +4645,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>8</v>
       </c>
@@ -4668,7 +4668,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>8</v>
       </c>
@@ -4691,7 +4691,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>8</v>
       </c>
@@ -4714,7 +4714,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>8</v>
       </c>
@@ -4737,7 +4737,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>8</v>
       </c>
@@ -4760,7 +4760,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="31" spans="1:7">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>8</v>
       </c>
@@ -4783,7 +4783,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="32" spans="1:7">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>8</v>
       </c>
@@ -4806,7 +4806,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="33" spans="1:7">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>8</v>
       </c>
@@ -4829,7 +4829,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>8</v>
       </c>
@@ -4852,7 +4852,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>8</v>
       </c>
@@ -4875,7 +4875,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -4898,7 +4898,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>8</v>
       </c>
@@ -4921,7 +4921,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>8</v>
       </c>
@@ -4944,7 +4944,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>8</v>
       </c>
@@ -4967,7 +4967,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>8</v>
       </c>
@@ -4990,7 +4990,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>8</v>
       </c>
@@ -5013,7 +5013,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>8</v>
       </c>
@@ -5036,7 +5036,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="43" spans="1:7">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>8</v>
       </c>
@@ -5059,7 +5059,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>8</v>
       </c>
@@ -5082,7 +5082,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="45" spans="1:7">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>8</v>
       </c>
@@ -5105,7 +5105,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>8</v>
       </c>
@@ -5128,7 +5128,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="47" spans="1:7">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>8</v>
       </c>
@@ -5151,7 +5151,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="48" spans="1:7">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>8</v>
       </c>
@@ -5174,7 +5174,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="49" spans="1:7">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>8</v>
       </c>
@@ -5197,7 +5197,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="50" spans="1:7">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>8</v>
       </c>
@@ -5220,7 +5220,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="51" spans="1:7">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>8</v>
       </c>
@@ -5243,7 +5243,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="52" spans="1:7">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>8</v>
       </c>
@@ -5266,7 +5266,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="53" spans="1:7">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>8</v>
       </c>
@@ -5289,7 +5289,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="54" spans="1:7">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>8</v>
       </c>
@@ -5312,7 +5312,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="55" spans="1:7">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>8</v>
       </c>
@@ -5335,7 +5335,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="56" spans="1:7">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>8</v>
       </c>
@@ -5358,7 +5358,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="57" spans="1:7">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>8</v>
       </c>
@@ -5381,7 +5381,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="58" spans="1:7">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>8</v>
       </c>
@@ -5404,7 +5404,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="59" spans="1:7">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>8</v>
       </c>
@@ -5427,7 +5427,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="60" spans="1:7">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>8</v>
       </c>
@@ -5450,7 +5450,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="61" spans="1:7">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>8</v>
       </c>
@@ -5473,7 +5473,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="62" spans="1:7">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>8</v>
       </c>
@@ -5496,7 +5496,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="63" spans="1:7">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>8</v>
       </c>
@@ -5519,7 +5519,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="64" spans="1:7">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>8</v>
       </c>
@@ -5542,7 +5542,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="65" spans="1:7">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>8</v>
       </c>
@@ -5565,7 +5565,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="66" spans="1:7">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>8</v>
       </c>
@@ -5588,7 +5588,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="67" spans="1:7">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>8</v>
       </c>
@@ -5611,7 +5611,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="68" spans="1:7">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>8</v>
       </c>
@@ -5634,7 +5634,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="69" spans="1:7">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>8</v>
       </c>
@@ -5657,7 +5657,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="70" spans="1:7">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>8</v>
       </c>
@@ -5680,7 +5680,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="71" spans="1:7">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>8</v>
       </c>
@@ -5703,7 +5703,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="72" spans="1:7">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>8</v>
       </c>
@@ -5726,7 +5726,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="73" spans="1:7">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>8</v>
       </c>
@@ -5749,7 +5749,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="74" spans="1:7">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>8</v>
       </c>
@@ -5772,7 +5772,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="75" spans="1:7">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>8</v>
       </c>
@@ -5795,7 +5795,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="76" spans="1:7">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>8</v>
       </c>
@@ -5818,7 +5818,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="77" spans="1:7">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>8</v>
       </c>
@@ -5841,7 +5841,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="78" spans="1:7">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -5864,7 +5864,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="79" spans="1:7">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>8</v>
       </c>
@@ -5887,7 +5887,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="80" spans="1:7">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>8</v>
       </c>
@@ -5910,7 +5910,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="81" spans="1:7">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>8</v>
       </c>
@@ -5933,7 +5933,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="82" spans="1:7">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>8</v>
       </c>
@@ -5956,7 +5956,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="83" spans="1:7">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>8</v>
       </c>
@@ -5979,7 +5979,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="84" spans="1:7">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>8</v>
       </c>
@@ -6002,7 +6002,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="85" spans="1:7">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>8</v>
       </c>
@@ -6025,7 +6025,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="86" spans="1:7">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>8</v>
       </c>
@@ -6048,7 +6048,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="87" spans="1:7">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>8</v>
       </c>
@@ -6071,7 +6071,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="88" spans="1:7">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>8</v>
       </c>
@@ -6094,7 +6094,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="89" spans="1:7">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>8</v>
       </c>
@@ -6117,7 +6117,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="90" spans="1:7">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>8</v>
       </c>
@@ -6140,7 +6140,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="91" spans="1:7">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>8</v>
       </c>
@@ -6163,7 +6163,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="92" spans="1:7">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>8</v>
       </c>
@@ -6186,7 +6186,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="93" spans="1:7">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>8</v>
       </c>
@@ -6209,7 +6209,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="94" spans="1:7">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>8</v>
       </c>
@@ -6232,7 +6232,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="95" spans="1:7">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>8</v>
       </c>
@@ -6255,7 +6255,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="96" spans="1:7">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>8</v>
       </c>
@@ -6278,7 +6278,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="97" spans="1:7">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>8</v>
       </c>
@@ -6301,7 +6301,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="98" spans="1:7">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>8</v>
       </c>
@@ -6324,7 +6324,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="99" spans="1:7">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>8</v>
       </c>
@@ -6347,7 +6347,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="100" spans="1:7">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>8</v>
       </c>
@@ -6370,7 +6370,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="101" spans="1:7">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>8</v>
       </c>
@@ -6393,7 +6393,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="102" spans="1:7">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>8</v>
       </c>
@@ -6416,7 +6416,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="103" spans="1:7">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>8</v>
       </c>
@@ -6439,7 +6439,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="104" spans="1:7">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>6</v>
       </c>
@@ -6462,7 +6462,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="105" spans="1:7">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>6</v>
       </c>
@@ -6485,7 +6485,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="106" spans="1:7">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>8</v>
       </c>
@@ -6508,7 +6508,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="107" spans="1:7">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>6</v>
       </c>
@@ -6531,7 +6531,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="108" spans="1:7">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>8</v>
       </c>
@@ -6554,7 +6554,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="109" spans="1:7">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>8</v>
       </c>
@@ -6588,7 +6588,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F214"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.33203125" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -6596,7 +6596,7 @@
     <col min="6" max="6" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6616,7 +6616,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -6636,7 +6636,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -6656,7 +6656,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -6676,7 +6676,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -6696,7 +6696,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -6716,7 +6716,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -6736,7 +6736,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -6756,7 +6756,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -6776,7 +6776,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -6796,7 +6796,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -6816,7 +6816,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -6836,7 +6836,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -6856,7 +6856,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -6876,7 +6876,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -6896,7 +6896,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -6916,7 +6916,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -6936,7 +6936,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -6956,7 +6956,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>8</v>
       </c>
@@ -6976,7 +6976,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>8</v>
       </c>
@@ -6996,7 +6996,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -7016,7 +7016,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>8</v>
       </c>
@@ -7036,7 +7036,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -7056,7 +7056,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>8</v>
       </c>
@@ -7076,7 +7076,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>8</v>
       </c>
@@ -7096,7 +7096,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>8</v>
       </c>
@@ -7116,7 +7116,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>8</v>
       </c>
@@ -7136,7 +7136,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>8</v>
       </c>
@@ -7156,7 +7156,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>8</v>
       </c>
@@ -7176,7 +7176,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>8</v>
       </c>
@@ -7196,7 +7196,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>8</v>
       </c>
@@ -7216,7 +7216,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>8</v>
       </c>
@@ -7236,7 +7236,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>8</v>
       </c>
@@ -7256,7 +7256,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>8</v>
       </c>
@@ -7276,7 +7276,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>8</v>
       </c>
@@ -7296,7 +7296,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -7316,7 +7316,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>8</v>
       </c>
@@ -7336,7 +7336,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>8</v>
       </c>
@@ -7356,7 +7356,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>8</v>
       </c>
@@ -7376,7 +7376,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>8</v>
       </c>
@@ -7396,7 +7396,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>8</v>
       </c>
@@ -7416,7 +7416,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>8</v>
       </c>
@@ -7436,7 +7436,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>8</v>
       </c>
@@ -7456,7 +7456,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="44" spans="1:6">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>8</v>
       </c>
@@ -7476,7 +7476,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>8</v>
       </c>
@@ -7496,7 +7496,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>8</v>
       </c>
@@ -7516,7 +7516,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>8</v>
       </c>
@@ -7536,7 +7536,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="48" spans="1:6">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>8</v>
       </c>
@@ -7556,7 +7556,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="49" spans="1:6">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>8</v>
       </c>
@@ -7576,7 +7576,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="50" spans="1:6">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>8</v>
       </c>
@@ -7596,7 +7596,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="51" spans="1:6">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>8</v>
       </c>
@@ -7616,7 +7616,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="52" spans="1:6">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>8</v>
       </c>
@@ -7636,7 +7636,7 @@
         <v>702</v>
       </c>
     </row>
-    <row r="53" spans="1:6">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>8</v>
       </c>
@@ -7656,7 +7656,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="54" spans="1:6">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>8</v>
       </c>
@@ -7676,7 +7676,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="55" spans="1:6">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>8</v>
       </c>
@@ -7696,7 +7696,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="56" spans="1:6">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>8</v>
       </c>
@@ -7716,7 +7716,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="57" spans="1:6">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>8</v>
       </c>
@@ -7736,7 +7736,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="58" spans="1:6">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>8</v>
       </c>
@@ -7756,7 +7756,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="59" spans="1:6">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>8</v>
       </c>
@@ -7776,7 +7776,7 @@
         <v>723</v>
       </c>
     </row>
-    <row r="60" spans="1:6">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>8</v>
       </c>
@@ -7796,7 +7796,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="61" spans="1:6">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>8</v>
       </c>
@@ -7816,7 +7816,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="62" spans="1:6">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>8</v>
       </c>
@@ -7836,7 +7836,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="63" spans="1:6">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>8</v>
       </c>
@@ -7856,7 +7856,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="64" spans="1:6">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>8</v>
       </c>
@@ -7876,7 +7876,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="65" spans="1:6">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>8</v>
       </c>
@@ -7896,7 +7896,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="66" spans="1:6">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>8</v>
       </c>
@@ -7916,7 +7916,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="67" spans="1:6">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>8</v>
       </c>
@@ -7936,7 +7936,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="68" spans="1:6">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>8</v>
       </c>
@@ -7956,7 +7956,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="69" spans="1:6">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>8</v>
       </c>
@@ -7976,7 +7976,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="70" spans="1:6">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>8</v>
       </c>
@@ -7996,7 +7996,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="71" spans="1:6">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>8</v>
       </c>
@@ -8016,7 +8016,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="72" spans="1:6">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>8</v>
       </c>
@@ -8036,7 +8036,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="73" spans="1:6">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>8</v>
       </c>
@@ -8056,7 +8056,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="74" spans="1:6">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>8</v>
       </c>
@@ -8076,7 +8076,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="75" spans="1:6">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>8</v>
       </c>
@@ -8096,7 +8096,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="76" spans="1:6">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>8</v>
       </c>
@@ -8116,7 +8116,7 @@
         <v>774</v>
       </c>
     </row>
-    <row r="77" spans="1:6">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>8</v>
       </c>
@@ -8136,7 +8136,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="78" spans="1:6">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -8156,7 +8156,7 @@
         <v>780</v>
       </c>
     </row>
-    <row r="79" spans="1:6">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>8</v>
       </c>
@@ -8176,7 +8176,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="80" spans="1:6">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>8</v>
       </c>
@@ -8196,7 +8196,7 @@
         <v>786</v>
       </c>
     </row>
-    <row r="81" spans="1:6">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>8</v>
       </c>
@@ -8216,7 +8216,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="82" spans="1:6">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>8</v>
       </c>
@@ -8236,7 +8236,7 @@
         <v>792</v>
       </c>
     </row>
-    <row r="83" spans="1:6">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>8</v>
       </c>
@@ -8256,7 +8256,7 @@
         <v>795</v>
       </c>
     </row>
-    <row r="84" spans="1:6">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>8</v>
       </c>
@@ -8276,7 +8276,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="85" spans="1:6">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>8</v>
       </c>
@@ -8296,7 +8296,7 @@
         <v>801</v>
       </c>
     </row>
-    <row r="86" spans="1:6">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>8</v>
       </c>
@@ -8316,7 +8316,7 @@
         <v>804</v>
       </c>
     </row>
-    <row r="87" spans="1:6">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>8</v>
       </c>
@@ -8336,7 +8336,7 @@
         <v>807</v>
       </c>
     </row>
-    <row r="88" spans="1:6">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>8</v>
       </c>
@@ -8356,7 +8356,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="89" spans="1:6">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>8</v>
       </c>
@@ -8376,7 +8376,7 @@
         <v>813</v>
       </c>
     </row>
-    <row r="90" spans="1:6">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>8</v>
       </c>
@@ -8396,7 +8396,7 @@
         <v>816</v>
       </c>
     </row>
-    <row r="91" spans="1:6">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>8</v>
       </c>
@@ -8416,7 +8416,7 @@
         <v>819</v>
       </c>
     </row>
-    <row r="92" spans="1:6">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>8</v>
       </c>
@@ -8436,7 +8436,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="93" spans="1:6">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>8</v>
       </c>
@@ -8456,7 +8456,7 @@
         <v>825</v>
       </c>
     </row>
-    <row r="94" spans="1:6">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>8</v>
       </c>
@@ -8476,7 +8476,7 @@
         <v>828</v>
       </c>
     </row>
-    <row r="95" spans="1:6">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>8</v>
       </c>
@@ -8496,7 +8496,7 @@
         <v>831</v>
       </c>
     </row>
-    <row r="96" spans="1:6">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>8</v>
       </c>
@@ -8516,7 +8516,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="97" spans="1:6">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>8</v>
       </c>
@@ -8536,7 +8536,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="98" spans="1:6">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>8</v>
       </c>
@@ -8556,7 +8556,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="99" spans="1:6">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>8</v>
       </c>
@@ -8576,7 +8576,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="100" spans="1:6">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>8</v>
       </c>
@@ -8596,7 +8596,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="101" spans="1:6">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>8</v>
       </c>
@@ -8616,7 +8616,7 @@
         <v>849</v>
       </c>
     </row>
-    <row r="102" spans="1:6">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>8</v>
       </c>
@@ -8636,7 +8636,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="103" spans="1:6">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>8</v>
       </c>
@@ -8656,7 +8656,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="104" spans="1:6">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>8</v>
       </c>
@@ -8676,7 +8676,7 @@
         <v>858</v>
       </c>
     </row>
-    <row r="105" spans="1:6">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>8</v>
       </c>
@@ -8696,7 +8696,7 @@
         <v>861</v>
       </c>
     </row>
-    <row r="106" spans="1:6">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>8</v>
       </c>
@@ -8716,7 +8716,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="107" spans="1:6">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>8</v>
       </c>
@@ -8736,7 +8736,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="108" spans="1:6">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>8</v>
       </c>
@@ -8756,7 +8756,7 @@
         <v>870</v>
       </c>
     </row>
-    <row r="109" spans="1:6">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>8</v>
       </c>
@@ -8776,7 +8776,7 @@
         <v>873</v>
       </c>
     </row>
-    <row r="110" spans="1:6">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>8</v>
       </c>
@@ -8796,7 +8796,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="111" spans="1:6">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>8</v>
       </c>
@@ -8816,7 +8816,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="112" spans="1:6">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>8</v>
       </c>
@@ -8836,7 +8836,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="113" spans="1:6">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>8</v>
       </c>
@@ -8856,7 +8856,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="114" spans="1:6">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>8</v>
       </c>
@@ -8876,7 +8876,7 @@
         <v>888</v>
       </c>
     </row>
-    <row r="115" spans="1:6">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>8</v>
       </c>
@@ -8896,7 +8896,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="116" spans="1:6">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>8</v>
       </c>
@@ -8916,7 +8916,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="117" spans="1:6">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>8</v>
       </c>
@@ -8936,7 +8936,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="118" spans="1:6">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>8</v>
       </c>
@@ -8956,7 +8956,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="119" spans="1:6">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>8</v>
       </c>
@@ -8976,7 +8976,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="120" spans="1:6">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>8</v>
       </c>
@@ -8996,7 +8996,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="121" spans="1:6">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>8</v>
       </c>
@@ -9016,7 +9016,7 @@
         <v>909</v>
       </c>
     </row>
-    <row r="122" spans="1:6">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>8</v>
       </c>
@@ -9036,7 +9036,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="123" spans="1:6">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>8</v>
       </c>
@@ -9056,7 +9056,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="124" spans="1:6">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>8</v>
       </c>
@@ -9076,7 +9076,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="125" spans="1:6">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>8</v>
       </c>
@@ -9096,7 +9096,7 @@
         <v>921</v>
       </c>
     </row>
-    <row r="126" spans="1:6">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>8</v>
       </c>
@@ -9116,7 +9116,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="127" spans="1:6">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>8</v>
       </c>
@@ -9136,7 +9136,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="128" spans="1:6">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>8</v>
       </c>
@@ -9156,7 +9156,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="129" spans="1:6">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>8</v>
       </c>
@@ -9176,7 +9176,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="130" spans="1:6">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>8</v>
       </c>
@@ -9196,7 +9196,7 @@
         <v>936</v>
       </c>
     </row>
-    <row r="131" spans="1:6">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>8</v>
       </c>
@@ -9216,7 +9216,7 @@
         <v>939</v>
       </c>
     </row>
-    <row r="132" spans="1:6">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>8</v>
       </c>
@@ -9236,7 +9236,7 @@
         <v>942</v>
       </c>
     </row>
-    <row r="133" spans="1:6">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>8</v>
       </c>
@@ -9256,7 +9256,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="134" spans="1:6">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>8</v>
       </c>
@@ -9276,7 +9276,7 @@
         <v>948</v>
       </c>
     </row>
-    <row r="135" spans="1:6">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>8</v>
       </c>
@@ -9296,7 +9296,7 @@
         <v>951</v>
       </c>
     </row>
-    <row r="136" spans="1:6">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>8</v>
       </c>
@@ -9316,7 +9316,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="137" spans="1:6">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>8</v>
       </c>
@@ -9336,7 +9336,7 @@
         <v>957</v>
       </c>
     </row>
-    <row r="138" spans="1:6">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>8</v>
       </c>
@@ -9356,7 +9356,7 @@
         <v>960</v>
       </c>
     </row>
-    <row r="139" spans="1:6">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>8</v>
       </c>
@@ -9376,7 +9376,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="140" spans="1:6">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>8</v>
       </c>
@@ -9396,7 +9396,7 @@
         <v>966</v>
       </c>
     </row>
-    <row r="141" spans="1:6">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>8</v>
       </c>
@@ -9416,7 +9416,7 @@
         <v>969</v>
       </c>
     </row>
-    <row r="142" spans="1:6">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>8</v>
       </c>
@@ -9436,7 +9436,7 @@
         <v>972</v>
       </c>
     </row>
-    <row r="143" spans="1:6">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>8</v>
       </c>
@@ -9456,7 +9456,7 @@
         <v>975</v>
       </c>
     </row>
-    <row r="144" spans="1:6">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>8</v>
       </c>
@@ -9476,7 +9476,7 @@
         <v>978</v>
       </c>
     </row>
-    <row r="145" spans="1:6">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>8</v>
       </c>
@@ -9496,7 +9496,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="146" spans="1:6">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>8</v>
       </c>
@@ -9516,7 +9516,7 @@
         <v>984</v>
       </c>
     </row>
-    <row r="147" spans="1:6">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>8</v>
       </c>
@@ -9536,7 +9536,7 @@
         <v>987</v>
       </c>
     </row>
-    <row r="148" spans="1:6">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>8</v>
       </c>
@@ -9556,7 +9556,7 @@
         <v>991</v>
       </c>
     </row>
-    <row r="149" spans="1:6">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>8</v>
       </c>
@@ -9576,7 +9576,7 @@
         <v>994</v>
       </c>
     </row>
-    <row r="150" spans="1:6">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>8</v>
       </c>
@@ -9596,7 +9596,7 @@
         <v>997</v>
       </c>
     </row>
-    <row r="151" spans="1:6">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>8</v>
       </c>
@@ -9616,7 +9616,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="152" spans="1:6">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>8</v>
       </c>
@@ -9636,7 +9636,7 @@
         <v>1003</v>
       </c>
     </row>
-    <row r="153" spans="1:6">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>8</v>
       </c>
@@ -9656,7 +9656,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="154" spans="1:6">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>8</v>
       </c>
@@ -9676,7 +9676,7 @@
         <v>1009</v>
       </c>
     </row>
-    <row r="155" spans="1:6">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>8</v>
       </c>
@@ -9696,7 +9696,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="156" spans="1:6">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>8</v>
       </c>
@@ -9716,7 +9716,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="157" spans="1:6">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>8</v>
       </c>
@@ -9736,7 +9736,7 @@
         <v>1018</v>
       </c>
     </row>
-    <row r="158" spans="1:6">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>8</v>
       </c>
@@ -9756,7 +9756,7 @@
         <v>1021</v>
       </c>
     </row>
-    <row r="159" spans="1:6">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>8</v>
       </c>
@@ -9776,7 +9776,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="160" spans="1:6">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>8</v>
       </c>
@@ -9796,7 +9796,7 @@
         <v>1027</v>
       </c>
     </row>
-    <row r="161" spans="1:6">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>8</v>
       </c>
@@ -9816,7 +9816,7 @@
         <v>1030</v>
       </c>
     </row>
-    <row r="162" spans="1:6">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>8</v>
       </c>
@@ -9836,7 +9836,7 @@
         <v>1033</v>
       </c>
     </row>
-    <row r="163" spans="1:6">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>8</v>
       </c>
@@ -9856,7 +9856,7 @@
         <v>1036</v>
       </c>
     </row>
-    <row r="164" spans="1:6">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>8</v>
       </c>
@@ -9876,7 +9876,7 @@
         <v>1039</v>
       </c>
     </row>
-    <row r="165" spans="1:6">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>8</v>
       </c>
@@ -9896,7 +9896,7 @@
         <v>1042</v>
       </c>
     </row>
-    <row r="166" spans="1:6">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>8</v>
       </c>
@@ -9916,7 +9916,7 @@
         <v>1045</v>
       </c>
     </row>
-    <row r="167" spans="1:6">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>8</v>
       </c>
@@ -9936,7 +9936,7 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="168" spans="1:6">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>8</v>
       </c>
@@ -9956,7 +9956,7 @@
         <v>1051</v>
       </c>
     </row>
-    <row r="169" spans="1:6">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>8</v>
       </c>
@@ -9976,7 +9976,7 @@
         <v>1054</v>
       </c>
     </row>
-    <row r="170" spans="1:6">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>8</v>
       </c>
@@ -9996,7 +9996,7 @@
         <v>1057</v>
       </c>
     </row>
-    <row r="171" spans="1:6">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>8</v>
       </c>
@@ -10016,7 +10016,7 @@
         <v>1060</v>
       </c>
     </row>
-    <row r="172" spans="1:6">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>8</v>
       </c>
@@ -10036,7 +10036,7 @@
         <v>1063</v>
       </c>
     </row>
-    <row r="173" spans="1:6">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>8</v>
       </c>
@@ -10056,7 +10056,7 @@
         <v>1066</v>
       </c>
     </row>
-    <row r="174" spans="1:6">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>8</v>
       </c>
@@ -10076,7 +10076,7 @@
         <v>1069</v>
       </c>
     </row>
-    <row r="175" spans="1:6">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>8</v>
       </c>
@@ -10096,7 +10096,7 @@
         <v>1072</v>
       </c>
     </row>
-    <row r="176" spans="1:6">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>8</v>
       </c>
@@ -10116,7 +10116,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="177" spans="1:6">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>8</v>
       </c>
@@ -10136,7 +10136,7 @@
         <v>1078</v>
       </c>
     </row>
-    <row r="178" spans="1:6">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>8</v>
       </c>
@@ -10156,7 +10156,7 @@
         <v>1081</v>
       </c>
     </row>
-    <row r="179" spans="1:6">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>8</v>
       </c>
@@ -10176,7 +10176,7 @@
         <v>1084</v>
       </c>
     </row>
-    <row r="180" spans="1:6">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>8</v>
       </c>
@@ -10196,7 +10196,7 @@
         <v>1087</v>
       </c>
     </row>
-    <row r="181" spans="1:6">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>8</v>
       </c>
@@ -10216,7 +10216,7 @@
         <v>1090</v>
       </c>
     </row>
-    <row r="182" spans="1:6">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>8</v>
       </c>
@@ -10236,7 +10236,7 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="183" spans="1:6">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>8</v>
       </c>
@@ -10256,7 +10256,7 @@
         <v>1096</v>
       </c>
     </row>
-    <row r="184" spans="1:6">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>8</v>
       </c>
@@ -10276,7 +10276,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="185" spans="1:6">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>8</v>
       </c>
@@ -10296,7 +10296,7 @@
         <v>1102</v>
       </c>
     </row>
-    <row r="186" spans="1:6">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>8</v>
       </c>
@@ -10316,7 +10316,7 @@
         <v>1105</v>
       </c>
     </row>
-    <row r="187" spans="1:6">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>8</v>
       </c>
@@ -10336,7 +10336,7 @@
         <v>1108</v>
       </c>
     </row>
-    <row r="188" spans="1:6">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>8</v>
       </c>
@@ -10356,7 +10356,7 @@
         <v>1111</v>
       </c>
     </row>
-    <row r="189" spans="1:6">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>8</v>
       </c>
@@ -10376,7 +10376,7 @@
         <v>1114</v>
       </c>
     </row>
-    <row r="190" spans="1:6">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>8</v>
       </c>
@@ -10396,7 +10396,7 @@
         <v>1117</v>
       </c>
     </row>
-    <row r="191" spans="1:6">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>8</v>
       </c>
@@ -10416,7 +10416,7 @@
         <v>1120</v>
       </c>
     </row>
-    <row r="192" spans="1:6">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>8</v>
       </c>
@@ -10436,7 +10436,7 @@
         <v>1123</v>
       </c>
     </row>
-    <row r="193" spans="1:6">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>8</v>
       </c>
@@ -10456,7 +10456,7 @@
         <v>1126</v>
       </c>
     </row>
-    <row r="194" spans="1:6">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>8</v>
       </c>
@@ -10476,7 +10476,7 @@
         <v>1129</v>
       </c>
     </row>
-    <row r="195" spans="1:6">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>8</v>
       </c>
@@ -10496,7 +10496,7 @@
         <v>1132</v>
       </c>
     </row>
-    <row r="196" spans="1:6">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>8</v>
       </c>
@@ -10516,7 +10516,7 @@
         <v>1135</v>
       </c>
     </row>
-    <row r="197" spans="1:6">
+    <row r="197" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>8</v>
       </c>
@@ -10536,7 +10536,7 @@
         <v>1138</v>
       </c>
     </row>
-    <row r="198" spans="1:6">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>8</v>
       </c>
@@ -10556,7 +10556,7 @@
         <v>1141</v>
       </c>
     </row>
-    <row r="199" spans="1:6">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>8</v>
       </c>
@@ -10576,7 +10576,7 @@
         <v>1144</v>
       </c>
     </row>
-    <row r="200" spans="1:6">
+    <row r="200" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>8</v>
       </c>
@@ -10596,7 +10596,7 @@
         <v>1147</v>
       </c>
     </row>
-    <row r="201" spans="1:6">
+    <row r="201" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>8</v>
       </c>
@@ -10616,7 +10616,7 @@
         <v>1150</v>
       </c>
     </row>
-    <row r="202" spans="1:6">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>8</v>
       </c>
@@ -10636,7 +10636,7 @@
         <v>1153</v>
       </c>
     </row>
-    <row r="203" spans="1:6">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>8</v>
       </c>
@@ -10656,7 +10656,7 @@
         <v>1156</v>
       </c>
     </row>
-    <row r="204" spans="1:6">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>8</v>
       </c>
@@ -10676,7 +10676,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="205" spans="1:6">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>8</v>
       </c>
@@ -10696,7 +10696,7 @@
         <v>1162</v>
       </c>
     </row>
-    <row r="206" spans="1:6">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>8</v>
       </c>
@@ -10716,7 +10716,7 @@
         <v>1165</v>
       </c>
     </row>
-    <row r="207" spans="1:6">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>8</v>
       </c>
@@ -10736,7 +10736,7 @@
         <v>1168</v>
       </c>
     </row>
-    <row r="208" spans="1:6">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>8</v>
       </c>
@@ -10756,7 +10756,7 @@
         <v>1171</v>
       </c>
     </row>
-    <row r="209" spans="1:6">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>8</v>
       </c>
@@ -10776,7 +10776,7 @@
         <v>1174</v>
       </c>
     </row>
-    <row r="210" spans="1:6">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>8</v>
       </c>
@@ -10796,7 +10796,7 @@
         <v>1177</v>
       </c>
     </row>
-    <row r="211" spans="1:6">
+    <row r="211" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>8</v>
       </c>
@@ -10816,7 +10816,7 @@
         <v>1180</v>
       </c>
     </row>
-    <row r="212" spans="1:6">
+    <row r="212" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>8</v>
       </c>
@@ -10836,7 +10836,7 @@
         <v>1183</v>
       </c>
     </row>
-    <row r="213" spans="1:6">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>8</v>
       </c>
@@ -10856,7 +10856,7 @@
         <v>1186</v>
       </c>
     </row>
-    <row r="214" spans="1:6">
+    <row r="214" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>8</v>
       </c>

</xml_diff>